<commit_message>
ajustes galería old, actualización docus gestión, docu, detalle patrimonio
</commit_message>
<xml_diff>
--- a/src/Documentacion/BIS011APPSY-SeguimientoPlanTrabajoDesaHERRIZ-v2.xlsx
+++ b/src/Documentacion/BIS011APPSY-SeguimientoPlanTrabajoDesaHERRIZ-v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sgantolin\BiscaytikApp_node-modules-incluido\src\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{935813E1-8E55-4825-AF0C-3C4ECC6F2759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8515182E-BAB6-4A59-BD51-5F4497A91540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="242">
   <si>
     <t>HITO</t>
   </si>
@@ -677,18 +677,12 @@
     <t>Falta estimar funcionalidad compartir.</t>
   </si>
   <si>
-    <t>pequeña corrección pendiente de entregar en listados</t>
-  </si>
-  <si>
     <t>Validación contenido? Ejem. Galería ? (reglas)</t>
   </si>
   <si>
     <t>si no hay contenido no aparece posible?  Estimar</t>
   </si>
   <si>
-    <t>Condicionado. Revisar tab galería</t>
-  </si>
-  <si>
     <t>img's SVGs para poder editarlas por css. Iconos "mejor elegidos"</t>
   </si>
   <si>
@@ -756,6 +750,18 @@
   </si>
   <si>
     <t>Condicionado. Consulta canal</t>
+  </si>
+  <si>
+    <t>Finalizado. Rehecho img 100%</t>
+  </si>
+  <si>
+    <t>En listados repetido por estructura sitio</t>
+  </si>
+  <si>
+    <t>Condicionado. Revisar tab galería?</t>
+  </si>
+  <si>
+    <t>En curso. 1ra prueba hecha.Cuando esté todo el portal revisar acad punto</t>
   </si>
 </sst>
 </file>
@@ -1034,7 +1040,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1180,6 +1186,9 @@
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1197,10 +1206,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1608,7 +1613,7 @@
         <v>180</v>
       </c>
       <c r="AD2" s="35" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="AE2" s="35" t="s">
         <v>181</v>
@@ -1876,10 +1881,10 @@
         <v>167</v>
       </c>
       <c r="AB15" s="19" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AD15" s="43" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="16" spans="1:32" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -1926,7 +1931,7 @@
         <v>184</v>
       </c>
       <c r="AA17" s="45" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="AD17" s="43" t="s">
         <v>166</v>
@@ -2287,7 +2292,7 @@
         <v>208</v>
       </c>
       <c r="AD30" s="44" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="31" spans="1:31" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -2403,7 +2408,7 @@
         <v>186</v>
       </c>
       <c r="AC35" s="19" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="AD35" s="46" t="s">
         <v>209</v>
@@ -2412,7 +2417,7 @@
         <v>186</v>
       </c>
       <c r="AF35" s="19" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="36" spans="1:32" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -2623,22 +2628,22 @@
       </c>
       <c r="X43" s="41"/>
       <c r="AA43" s="44" t="s">
+        <v>221</v>
+      </c>
+      <c r="AB43" s="54" t="s">
+        <v>224</v>
+      </c>
+      <c r="AC43" s="19" t="s">
         <v>223</v>
       </c>
-      <c r="AB43" s="54" t="s">
-        <v>226</v>
-      </c>
-      <c r="AC43" s="19" t="s">
-        <v>225</v>
-      </c>
       <c r="AD43" s="44" t="s">
+        <v>221</v>
+      </c>
+      <c r="AE43" s="54" t="s">
+        <v>224</v>
+      </c>
+      <c r="AF43" s="19" t="s">
         <v>223</v>
-      </c>
-      <c r="AE43" s="54" t="s">
-        <v>226</v>
-      </c>
-      <c r="AF43" s="19" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="44" spans="1:32" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -2671,7 +2676,7 @@
     </row>
     <row r="45" spans="1:32" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="50" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B45" s="16" t="s">
         <v>64</v>
@@ -2698,19 +2703,19 @@
         <v>210</v>
       </c>
       <c r="AB45" s="19" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="AC45" s="19" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="AD45" s="44" t="s">
         <v>210</v>
       </c>
       <c r="AE45" s="19" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="AF45" s="19" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="46" spans="1:32" ht="28.8" outlineLevel="2" x14ac:dyDescent="0.3">
@@ -3083,7 +3088,7 @@
         <v>212</v>
       </c>
       <c r="AC60" s="19" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AD60" s="43" t="s">
         <v>166</v>
@@ -3092,7 +3097,7 @@
         <v>212</v>
       </c>
       <c r="AF60" s="19" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="61" spans="1:32" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -3123,17 +3128,17 @@
       <c r="Y61" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="AA61" s="44" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB61" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="AD61" s="44" t="s">
-        <v>167</v>
-      </c>
-      <c r="AE61" s="19" t="s">
-        <v>213</v>
+      <c r="AA61" s="43" t="s">
+        <v>166</v>
+      </c>
+      <c r="AB61" s="55" t="s">
+        <v>239</v>
+      </c>
+      <c r="AD61" s="43" t="s">
+        <v>166</v>
+      </c>
+      <c r="AE61" s="55" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="62" spans="1:32" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -3183,7 +3188,7 @@
         <v>189</v>
       </c>
       <c r="AD62" s="43" t="s">
-        <v>166</v>
+        <v>238</v>
       </c>
       <c r="AE62" s="19" t="s">
         <v>190</v>
@@ -3265,16 +3270,16 @@
         <v>193</v>
       </c>
       <c r="AA64" s="44" t="s">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="AB64" s="19" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AD64" s="44" t="s">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="AE64" s="19" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="65" spans="1:32" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -3432,7 +3437,7 @@
         <v>145</v>
       </c>
       <c r="X69" s="37" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="Y69" s="19" t="s">
         <v>194</v>
@@ -3441,7 +3446,7 @@
         <v>202</v>
       </c>
       <c r="AA69" s="46" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="AB69" s="19" t="s">
         <v>194</v>
@@ -3450,7 +3455,7 @@
         <v>202</v>
       </c>
       <c r="AD69" s="46" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="AE69" s="19" t="s">
         <v>194</v>
@@ -3475,10 +3480,10 @@
     </row>
     <row r="71" spans="1:32" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A71" s="49" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C71" s="27" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D71" s="34" t="s">
         <v>92</v>
@@ -3517,10 +3522,10 @@
     </row>
     <row r="72" spans="1:32" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A72" s="49" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C72" s="27" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D72" s="13" t="s">
         <v>94</v>
@@ -3560,16 +3565,16 @@
         <v>169</v>
       </c>
       <c r="AB72" s="19" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="AC72" s="19" t="s">
         <v>197</v>
       </c>
-      <c r="AD72" s="46" t="s">
-        <v>169</v>
+      <c r="AD72" s="45" t="s">
+        <v>241</v>
       </c>
       <c r="AE72" s="19" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="AF72" s="19" t="s">
         <v>197</v>
@@ -3619,13 +3624,13 @@
         <v>169</v>
       </c>
       <c r="AB73" s="19" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="AD73" s="46" t="s">
         <v>169</v>
       </c>
       <c r="AE73" s="19" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="74" spans="1:32" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -3660,13 +3665,13 @@
         <v>169</v>
       </c>
       <c r="AB74" s="19" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="AD74" s="46" t="s">
         <v>169</v>
       </c>
       <c r="AE74" s="19" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="75" spans="1:32" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -3700,13 +3705,13 @@
         <v>167</v>
       </c>
       <c r="AC75" s="19" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="AD75" s="44" t="s">
         <v>167</v>
       </c>
       <c r="AF75" s="19" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="76" spans="1:32" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -3743,13 +3748,13 @@
         <v>169</v>
       </c>
       <c r="AB76" s="19" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AD76" s="46" t="s">
         <v>169</v>
       </c>
       <c r="AE76" s="19" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="77" spans="1:32" ht="63" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -3966,24 +3971,24 @@
         <v>169</v>
       </c>
       <c r="AB81" s="19" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="AC81" s="19" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="AD81" s="46" t="s">
         <v>169</v>
       </c>
       <c r="AE81" s="19" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="AF81" s="19" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="82" spans="1:32" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A82" s="50" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B82" s="16" t="s">
         <v>112</v>
@@ -4177,7 +4182,7 @@
     </row>
     <row r="91" spans="1:32" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A91" s="50" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B91" s="16" t="s">
         <v>125</v>
@@ -4347,38 +4352,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Estado xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">En curso</Estado>
-    <Area xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">7</Area>
-    <Acciones xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <sys xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <Sociedad xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <fechadeproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">2022-07-13T22:00:00+00:00</fechadeproyecto>
-    <OfertaAnterior xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Oferta xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
-      <Value>5919</Value>
-    </Oferta>
-    <responsableproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
-      <UserInfo>
-        <DisplayName>Aitor Roncero Val</DisplayName>
-        <AccountId>927</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </responsableproyecto>
-    <Oficina xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">1</Oficina>
-    <codigodeproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">Maquetación de páginas web dentro del proyecto Biscaytik</codigodeproyecto>
-    <fechafinestimado xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <TaxCatchAll xmlns="06fec347-a373-485e-bb4f-f611040a1dd3" xsi:nil="true"/>
-    <Cliente xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">209</Cliente>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <fechafinreal xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <Oferta_x0020_Antigua xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4782,28 +4761,44 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Estado xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">En curso</Estado>
+    <Area xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">7</Area>
+    <Acciones xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <sys xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <Sociedad xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <fechadeproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">2022-07-13T22:00:00+00:00</fechadeproyecto>
+    <OfertaAnterior xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Oferta xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
+      <Value>5919</Value>
+    </Oferta>
+    <responsableproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
+      <UserInfo>
+        <DisplayName>Aitor Roncero Val</DisplayName>
+        <AccountId>927</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </responsableproyecto>
+    <Oficina xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">1</Oficina>
+    <codigodeproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">Maquetación de páginas web dentro del proyecto Biscaytik</codigodeproyecto>
+    <fechafinestimado xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <TaxCatchAll xmlns="06fec347-a373-485e-bb4f-f611040a1dd3" xsi:nil="true"/>
+    <Cliente xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">209</Cliente>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <fechafinreal xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <Oferta_x0020_Antigua xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C64067D8-2529-40F8-873F-7DCFF29E6C0A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5D2ED08-240E-422E-815D-BA2AE63D0B29}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="06fec347-a373-485e-bb4f-f611040a1dd3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4829,9 +4824,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5D2ED08-240E-422E-815D-BA2AE63D0B29}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C64067D8-2529-40F8-873F-7DCFF29E6C0A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="06fec347-a373-485e-bb4f-f611040a1dd3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ajustes css, docus, código banner
</commit_message>
<xml_diff>
--- a/src/Documentacion/BIS011APPSY-SeguimientoPlanTrabajoDesaHERRIZ-v2.xlsx
+++ b/src/Documentacion/BIS011APPSY-SeguimientoPlanTrabajoDesaHERRIZ-v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sgantolin\BiscaytikApp_node-modules-incluido\src\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8515182E-BAB6-4A59-BD51-5F4497A91540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A6D7E5-F515-4507-89DC-62D2DEF9BE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="249">
   <si>
     <t>HITO</t>
   </si>
@@ -749,9 +749,6 @@
     <t xml:space="preserve">ESTADO  (02-09 parta teknei) </t>
   </si>
   <si>
-    <t>Condicionado. Consulta canal</t>
-  </si>
-  <si>
     <t>Finalizado. Rehecho img 100%</t>
   </si>
   <si>
@@ -762,6 +759,30 @@
   </si>
   <si>
     <t>En curso. 1ra prueba hecha.Cuando esté todo el portal revisar acad punto</t>
+  </si>
+  <si>
+    <t>En curso. Seria interesante añadir badge subcategoría</t>
+  </si>
+  <si>
+    <t>Falta funcionalidad compartir, estimación modificar estructura muestra servicios</t>
+  </si>
+  <si>
+    <t>Estimación horas nuevo. Tema tabs</t>
+  </si>
+  <si>
+    <t>contenido. Añadir 1 "diapositiva" más para que se muestre a modo slider. Estimación actual. New BTS5</t>
+  </si>
+  <si>
+    <t>A la espera modificaciones y definición con DESA</t>
+  </si>
+  <si>
+    <t>Condicionado. 1 ejem para todos los tipos (todos contenidos)</t>
+  </si>
+  <si>
+    <t>Condicionado. Dependiente contenidos y decisiones BKTT (todos contenidos)</t>
+  </si>
+  <si>
+    <t>Bloqueado. desarrollado en detalle bar. VALIDACIón , casos de uso</t>
   </si>
 </sst>
 </file>
@@ -2291,8 +2312,8 @@
       <c r="AB30" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="AD30" s="44" t="s">
-        <v>237</v>
+      <c r="AD30" s="43" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="31" spans="1:31" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -2363,7 +2384,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="35" spans="1:32" ht="72" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:32" ht="86.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A35" s="13" t="s">
         <v>178</v>
       </c>
@@ -2414,7 +2435,7 @@
         <v>209</v>
       </c>
       <c r="AE35" s="19" t="s">
-        <v>186</v>
+        <v>244</v>
       </c>
       <c r="AF35" s="19" t="s">
         <v>234</v>
@@ -2594,7 +2615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:32" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:32" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A43" s="32" t="s">
         <v>62</v>
       </c>
@@ -2637,10 +2658,7 @@
         <v>223</v>
       </c>
       <c r="AD43" s="44" t="s">
-        <v>221</v>
-      </c>
-      <c r="AE43" s="54" t="s">
-        <v>224</v>
+        <v>246</v>
       </c>
       <c r="AF43" s="19" t="s">
         <v>223</v>
@@ -2674,7 +2692,7 @@
       <c r="AA44" s="47"/>
       <c r="AD44" s="47"/>
     </row>
-    <row r="45" spans="1:32" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:32" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A45" s="50" t="s">
         <v>222</v>
       </c>
@@ -2709,7 +2727,7 @@
         <v>223</v>
       </c>
       <c r="AD45" s="44" t="s">
-        <v>210</v>
+        <v>247</v>
       </c>
       <c r="AE45" s="19" t="s">
         <v>220</v>
@@ -2852,14 +2870,14 @@
       <c r="AB48" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="AD48" s="46" t="s">
-        <v>169</v>
+      <c r="AD48" s="45" t="s">
+        <v>168</v>
       </c>
       <c r="AE48" s="19" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="49" spans="1:32" outlineLevel="2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:32" ht="43.2" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A49" s="33" t="s">
         <v>172</v>
       </c>
@@ -2898,11 +2916,11 @@
       <c r="AB49" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="AD49" s="46" t="s">
-        <v>169</v>
-      </c>
-      <c r="AE49" s="19" t="s">
-        <v>183</v>
+      <c r="AD49" s="45" t="s">
+        <v>168</v>
+      </c>
+      <c r="AE49" s="55" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="50" spans="1:32" ht="23.4" x14ac:dyDescent="0.3">
@@ -3046,7 +3064,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:32" ht="57.6" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:32" ht="86.4" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="23" t="s">
+        <v>81</v>
+      </c>
       <c r="C60" s="23" t="s">
         <v>81</v>
       </c>
@@ -3093,8 +3114,8 @@
       <c r="AD60" s="43" t="s">
         <v>166</v>
       </c>
-      <c r="AE60" s="19" t="s">
-        <v>212</v>
+      <c r="AE60" s="55" t="s">
+        <v>242</v>
       </c>
       <c r="AF60" s="19" t="s">
         <v>213</v>
@@ -3132,13 +3153,13 @@
         <v>166</v>
       </c>
       <c r="AB61" s="55" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="AD61" s="43" t="s">
         <v>166</v>
       </c>
       <c r="AE61" s="55" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="62" spans="1:32" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -3188,10 +3209,10 @@
         <v>189</v>
       </c>
       <c r="AD62" s="43" t="s">
-        <v>238</v>
-      </c>
-      <c r="AE62" s="19" t="s">
-        <v>190</v>
+        <v>237</v>
+      </c>
+      <c r="AE62" s="55" t="s">
+        <v>243</v>
       </c>
       <c r="AF62" s="19" t="s">
         <v>189</v>
@@ -3270,13 +3291,13 @@
         <v>193</v>
       </c>
       <c r="AA64" s="44" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="AB64" s="19" t="s">
         <v>214</v>
       </c>
       <c r="AD64" s="44" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="AE64" s="19" t="s">
         <v>214</v>
@@ -3455,7 +3476,7 @@
         <v>202</v>
       </c>
       <c r="AD69" s="46" t="s">
-        <v>219</v>
+        <v>248</v>
       </c>
       <c r="AE69" s="19" t="s">
         <v>194</v>
@@ -3571,7 +3592,7 @@
         <v>197</v>
       </c>
       <c r="AD72" s="45" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AE72" s="19" t="s">
         <v>233</v>
@@ -3626,8 +3647,8 @@
       <c r="AB73" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="AD73" s="46" t="s">
-        <v>169</v>
+      <c r="AD73" s="45" t="s">
+        <v>241</v>
       </c>
       <c r="AE73" s="19" t="s">
         <v>232</v>

</xml_diff>

<commit_message>
ajustes wp banner / wrapper, imágenes para qué ver, docus etc.
</commit_message>
<xml_diff>
--- a/src/Documentacion/BIS011APPSY-SeguimientoPlanTrabajoDesaHERRIZ-v2.xlsx
+++ b/src/Documentacion/BIS011APPSY-SeguimientoPlanTrabajoDesaHERRIZ-v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sgantolin\BiscaytikApp_node-modules-incluido\src\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A6D7E5-F515-4507-89DC-62D2DEF9BE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA20F13E-2D77-4D22-A24A-EE86CCCBF7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3771,8 +3771,8 @@
       <c r="AB76" s="19" t="s">
         <v>230</v>
       </c>
-      <c r="AD76" s="46" t="s">
-        <v>169</v>
+      <c r="AD76" s="45" t="s">
+        <v>168</v>
       </c>
       <c r="AE76" s="19" t="s">
         <v>230</v>
@@ -4382,6 +4382,41 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Estado xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">En curso</Estado>
+    <Area xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">7</Area>
+    <Acciones xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <sys xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <Sociedad xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <fechadeproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">2022-07-13T22:00:00+00:00</fechadeproyecto>
+    <OfertaAnterior xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Oferta xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
+      <Value>5919</Value>
+    </Oferta>
+    <responsableproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
+      <UserInfo>
+        <DisplayName>Aitor Roncero Val</DisplayName>
+        <AccountId>927</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </responsableproyecto>
+    <Oficina xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">1</Oficina>
+    <codigodeproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">Maquetación de páginas web dentro del proyecto Biscaytik</codigodeproyecto>
+    <fechafinestimado xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <TaxCatchAll xmlns="06fec347-a373-485e-bb4f-f611040a1dd3" xsi:nil="true"/>
+    <Cliente xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">209</Cliente>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <fechafinreal xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+    <Oferta_x0020_Antigua xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010021AB849DB9524648A8F6CDAE5A42EE85" ma:contentTypeVersion="54" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5cf342e325584cfc73779b32cd8516cb">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xmlns:ns3="06fec347-a373-485e-bb4f-f611040a1dd3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="97bec9e280156beb57af844d85b9963b" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -4781,41 +4816,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Estado xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">En curso</Estado>
-    <Area xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">7</Area>
-    <Acciones xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <sys xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <Sociedad xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <fechadeproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">2022-07-13T22:00:00+00:00</fechadeproyecto>
-    <OfertaAnterior xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Oferta xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
-      <Value>5919</Value>
-    </Oferta>
-    <responsableproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
-      <UserInfo>
-        <DisplayName>Aitor Roncero Val</DisplayName>
-        <AccountId>927</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </responsableproyecto>
-    <Oficina xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">1</Oficina>
-    <codigodeproyecto xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">Maquetación de páginas web dentro del proyecto Biscaytik</codigodeproyecto>
-    <fechafinestimado xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <TaxCatchAll xmlns="06fec347-a373-485e-bb4f-f611040a1dd3" xsi:nil="true"/>
-    <Cliente xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">209</Cliente>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <fechafinreal xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-    <Oferta_x0020_Antigua xmlns="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5D2ED08-240E-422E-815D-BA2AE63D0B29}">
   <ds:schemaRefs>
@@ -4825,6 +4825,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C64067D8-2529-40F8-873F-7DCFF29E6C0A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="06fec347-a373-485e-bb4f-f611040a1dd3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B271E1E9-4B5A-43C8-93E9-EF9A1A456C27}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4842,22 +4860,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C64067D8-2529-40F8-873F-7DCFF29E6C0A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="06fec347-a373-485e-bb4f-f611040a1dd3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>